<commit_message>
Ship W3.8 replication and deterministic reproduction package
</commit_message>
<xml_diff>
--- a/docs/additional_files/Additional_file_3_gc_bin_ablation.xlsx
+++ b/docs/additional_files/Additional_file_3_gc_bin_ablation.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seed_details" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Athaliana_replication" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Athaliana_replication_phase2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Athaliana_replication_summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,8 +33,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +47,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,9 +67,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1388,4 +1405,1196 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>cohort</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>species</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>gc_bins</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>gc_pearson_r</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>delta_vs_1bin</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.9653206901202074</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.1275155287198362</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.8378051614003712</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.9671202757951874</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.182201312299787</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.7849189634954005</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.9472734042198386</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.2336874661154935</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.7135859381043451</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>confirmation</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.9774599118175736</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.3353017959806649</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>confirmation</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.6421581158369087</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>confirmation</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.9459997192684872</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.2816405950038157</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>confirmation</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.6643591242646716</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>confirmation</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.953593878947893</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.09411613553893039</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>confirmation</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0.8594777434089627</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>primary_new_cohort</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>mean_delta_r</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0.237019508841137</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>sd_delta_r</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0.1266329802951499</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>ci95_low</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>-0.07755425305748287</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>ci95_high</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0.5515932707397568</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>paired_t</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>3.241887150890925</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>paired_t_p</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0.08341625886548082</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>wilcoxon_p</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>replication_supported</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>mean_gc_mad_1bin</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0.04414412957328984</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>mean_gc_mad_5bin</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0.04486332771316078</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>mean_delta_gc_mad</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0.0007191981398709454</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>combined_sensitivity</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>mean_delta_r</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0.209077138943088</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>sd_delta_r</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0.09208086231886088</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>ci95_low</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0.1124442002733202</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>ci95_high</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0.3057100776128557</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>paired_t</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>5.561767064236621</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>paired_t_p</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0.002585040797303837</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>wilcoxon_p</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>cohort</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>species</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>gc_bins</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>gc_pearson_r</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>delta_vs_1bin</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.9225404294518975</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.3307495033952389</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.5917909260566586</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.9450109537197484</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.3810403144215787</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.5639706392981697</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>99</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.9631224313630666</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.4302173141913821</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>99</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.5329051171716845</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.949038275349619</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.3387340768179975</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.6103041985316215</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>122</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.9859976154825475</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.2686420085565827</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>122</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.7173556069259648</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>133</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.9818929231959272</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.05514031096282346</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>phase2</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>A. thaliana</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>133</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0.9267526122331038</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>cohort</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>seeds</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>mean_delta_r</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>sd_delta_r</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>ci95_low</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>ci95_high</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>paired_t_p</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>11,22,33</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.1811347690450389</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.05309400350767054</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.04924195266383019</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.3130275854262476</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.02746513371418006</v>
+      </c>
+      <c r="I2" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>first_replication</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>44,55,66</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.237019508841137</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.1266329802951499</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>-0.0775542530613812</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.5515932707436552</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.08341625886548083</v>
+      </c>
+      <c r="I3" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>second_replication</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>77,88,99,111,122,133</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.3007539213909339</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.1318378721769491</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.1623985596403924</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.4391092831414755</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.002532278912588194</v>
+      </c>
+      <c r="I4" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>pooled_12_seed</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>11,22,33,44,55,66,77,88,99,111,122,133</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.2549155301670109</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.1185190610092363</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.1796121114308514</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.3302189489031704</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>1.276100928915394e-05</v>
+      </c>
+      <c r="I5" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>